<commit_message>
Changes of Coho plots for better visulaization
</commit_message>
<xml_diff>
--- a/End-of-season Historic escapement files/RbtObsQuart.xlsx
+++ b/End-of-season Historic escapement files/RbtObsQuart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\WCVI\ESCAPEMENT\Data_Requests\2025\Maa-nulth Coho discussions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\POURFARAJV\Documents\GitHub\Somass-escapement-plots\End-of-season Historic escapement files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C671BB2-AA0B-4578-8C77-5EB13654C731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB23D27-D5F8-45C0-8DDD-BB74E75E1417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16470" yWindow="5520" windowWidth="30705" windowHeight="12750" xr2:uid="{9741CDEF-CA83-433B-B122-CF325E3C93FC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9741CDEF-CA83-433B-B122-CF325E3C93FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -115,9 +115,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -155,7 +155,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -261,7 +261,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -403,7 +403,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -411,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A95F0ADD-87D8-4FDF-993F-BA2AD8FB626F}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
@@ -1039,22 +1039,6 @@
         <v>2056.8000000000002</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>2024</v>
-      </c>
-      <c r="B28">
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>2025</v>
-      </c>
-      <c r="B29">
-        <v>5.5E-2</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>